<commit_message>
fix: correct start/end time keys in Excel export, add README.md
</commit_message>
<xml_diff>
--- a/references/2026-06-11/viral-cut-2026-06-11.xlsx
+++ b/references/2026-06-11/viral-cut-2026-06-11.xlsx
@@ -506,8 +506,16 @@
           <t>รอดตายเฉย !</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr"/>
-      <c r="E2" s="2" t="inlineStr"/>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>00:25:00</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>00:25:22</t>
+        </is>
+      </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
           <t>【🔴 LIVE】Garena RoV Thailand - 006_ 16_05_2026 _ @P2O4N2CH @MidveilMIIKO @Amui-san @ครามไง (1).mp4</t>
@@ -533,8 +541,16 @@
           <t>วีทูปเบอร์ ไฟต์เดี่ยวจบเกม</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr"/>
-      <c r="E3" s="2" t="inlineStr"/>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>00:56:50</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>00:57:50</t>
+        </is>
+      </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
           <t>【🔴 LIVE】Garena RoV Thailand - 006_ 16_05_2026 _ @P2O4N2CH @MidveilMIIKO @Amui-san @ครามไง (1).mp4</t>
@@ -560,8 +576,16 @@
           <t>Reflex  ระดับ nailiu</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="2" t="inlineStr"/>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>01:10:35</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>01:11:50</t>
+        </is>
+      </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
           <t>【🔴 LIVE】Garena RoV Thailand - 006_ 16_05_2026 _ @P2O4N2CH @MidveilMIIKO @Amui-san @ครามไง (1).mp4</t>
@@ -587,8 +611,16 @@
           <t>ไฟต์กันชุลมุน = ระเบิดเป็นโกโก้คัน</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="2" t="inlineStr"/>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>01:24:00</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>01:25:30</t>
+        </is>
+      </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
           <t>【🔴 LIVE】Garena RoV Thailand - 006_ 16_05_2026 _ @P2O4N2CH @MidveilMIIKO @Amui-san @ครามไง (1).mp4</t>

</xml_diff>